<commit_message>
check for spaces and other invalid characters in file names
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_errors_test.xlsx
+++ b/spec/fixtures/batch_submission_manifest_errors_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/spec/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5FD756C-A380-0C4E-9646-2FC415B6D80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD27215-A2CE-764D-8931-59FD4D7C1FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="278">
   <si>
     <t>Field Section</t>
   </si>
@@ -450,6 +450,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Values for Controlled Vocabulary type fields must match one of the options provided in this row. Each Controlled Vocabulary option is listed as a short-hand term value and a longer length full text description of the option. </t>
     </r>
@@ -459,6 +460,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Controlled vocabulary option values must match short-hand term values! </t>
     </r>
@@ -467,6 +469,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>They can't match full text descriptions of options, that will produce an error on manifest submission. An example options list could look like this.
 FirstOpt: First Example Option
@@ -917,6 +920,9 @@
   </si>
   <si>
     <t>https://www.morphosource.org/banner_image.png</t>
+  </si>
+  <si>
+    <t>file with space.zip</t>
   </si>
 </sst>
 </file>
@@ -933,47 +939,56 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF272727"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF222222"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1344,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06ED7EC9-286B-1D49-A57D-A989376D77CC}">
-  <dimension ref="A1:CH15"/>
+  <dimension ref="A1:CH16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="3" max="3" width="47.33203125" bestFit="1" customWidth="1"/>
@@ -3896,6 +3911,141 @@
       <c r="CG15" s="26"/>
       <c r="CH15" s="26"/>
     </row>
+    <row r="16" spans="1:86" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="4"/>
+      <c r="C16" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>252</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>267</v>
+      </c>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26" t="s">
+        <v>261</v>
+      </c>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26" t="s">
+        <v>239</v>
+      </c>
+      <c r="P16" s="26" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q16" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="R16" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="S16" s="27"/>
+      <c r="T16" s="27"/>
+      <c r="U16" s="30"/>
+      <c r="V16" s="30"/>
+      <c r="W16" s="30"/>
+      <c r="X16" s="30"/>
+      <c r="Y16" s="27">
+        <v>1.5365230000000001E-2</v>
+      </c>
+      <c r="Z16" s="27">
+        <v>1.5365230000000001E-2</v>
+      </c>
+      <c r="AA16" s="27">
+        <v>1.5365230000000001E-2</v>
+      </c>
+      <c r="AB16" s="27"/>
+      <c r="AC16" s="27"/>
+      <c r="AD16" s="26" t="s">
+        <v>243</v>
+      </c>
+      <c r="AE16" s="27"/>
+      <c r="AF16" s="26"/>
+      <c r="AG16" s="26"/>
+      <c r="AH16" s="26"/>
+      <c r="AI16" s="26"/>
+      <c r="AJ16" s="26"/>
+      <c r="AK16" s="26"/>
+      <c r="AL16" s="26"/>
+      <c r="AM16" s="26"/>
+      <c r="AN16" s="26"/>
+      <c r="AO16" s="26"/>
+      <c r="AP16" s="26"/>
+      <c r="AQ16" s="26"/>
+      <c r="AR16" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="AS16" s="26"/>
+      <c r="AT16" s="26"/>
+      <c r="AU16" s="26"/>
+      <c r="AV16" s="26"/>
+      <c r="AW16" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="AX16" s="27"/>
+      <c r="AY16" s="27"/>
+      <c r="AZ16" s="27">
+        <v>0.200098</v>
+      </c>
+      <c r="BA16" s="26" t="s">
+        <v>245</v>
+      </c>
+      <c r="BB16" s="26" t="s">
+        <v>273</v>
+      </c>
+      <c r="BC16" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="BD16" s="30"/>
+      <c r="BE16" s="27">
+        <v>3</v>
+      </c>
+      <c r="BF16" s="27">
+        <v>1680</v>
+      </c>
+      <c r="BG16" s="27">
+        <v>70</v>
+      </c>
+      <c r="BH16" s="27">
+        <v>1.54E-2</v>
+      </c>
+      <c r="BI16" s="27">
+        <v>220</v>
+      </c>
+      <c r="BJ16" s="26"/>
+      <c r="BK16" s="30"/>
+      <c r="BL16" s="30"/>
+      <c r="BM16" s="30"/>
+      <c r="BN16" s="30"/>
+      <c r="BO16" s="30"/>
+      <c r="BP16" s="30"/>
+      <c r="BQ16" s="30"/>
+      <c r="BR16" s="30"/>
+      <c r="BS16" s="30"/>
+      <c r="BT16" s="30"/>
+      <c r="BU16" s="30"/>
+      <c r="BV16" s="30"/>
+      <c r="BW16" s="30"/>
+      <c r="BX16" s="30"/>
+      <c r="BY16" s="26"/>
+      <c r="BZ16" s="26"/>
+      <c r="CA16" s="26"/>
+      <c r="CB16" s="30"/>
+      <c r="CC16" s="30"/>
+      <c r="CD16" s="30"/>
+      <c r="CE16" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="CF16" s="26"/>
+      <c r="CG16" s="26"/>
+      <c r="CH16" s="26"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>